<commit_message>
Major Updates added big features
</commit_message>
<xml_diff>
--- a/tverse-main/tverse-ims/src/main/resources/static/product_upload_template.xlsx
+++ b/tverse-main/tverse-ims/src/main/resources/static/product_upload_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tverse\tverse-ims\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tverse\tverse-main\tverse-ims\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57217D68-BF45-4C65-87D8-D567F148F5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{991B635F-30A5-4FE6-AEF5-4E3F7FAB0AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="13372" xr2:uid="{664E4388-EF6C-4020-A0D0-D618DC38DEE4}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>SKU</t>
   </si>
@@ -126,10 +126,22 @@
     <t>(Useful for the Dashboard view of product)</t>
   </si>
   <si>
-    <t>Image URL</t>
-  </si>
-  <si>
     <t>(To show product photos in the Picklist later)</t>
+  </si>
+  <si>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>Regular Price </t>
+  </si>
+  <si>
+    <t>Sale Price</t>
+  </si>
+  <si>
+    <t>Parent Image</t>
+  </si>
+  <si>
+    <t>Variant Image</t>
   </si>
 </sst>
 </file>
@@ -172,7 +184,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -312,11 +324,65 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -326,61 +392,41 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
           <bgColor theme="2" tint="-9.9948118533890809E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -708,9 +754,12 @@
     <col min="9" max="9" width="18.921875" style="1" customWidth="1"/>
     <col min="10" max="10" width="21.53515625" style="1" customWidth="1"/>
     <col min="11" max="11" width="12" style="1" customWidth="1"/>
-    <col min="12" max="15" width="12" style="10" customWidth="1"/>
-    <col min="16" max="16" width="11.23046875" style="10" customWidth="1"/>
-    <col min="17" max="16384" width="9.23046875" style="11"/>
+    <col min="12" max="15" width="12" style="7" customWidth="1"/>
+    <col min="16" max="16" width="11.23046875" style="7" customWidth="1"/>
+    <col min="17" max="17" width="26.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="35.07421875" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="36.4609375" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="45.84375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="48" customHeight="1" x14ac:dyDescent="0.4">
@@ -732,90 +781,102 @@
       <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="O1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="P1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="Q1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="R1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="7" t="s">
-        <v>30</v>
+      <c r="S1" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="67.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="9"/>
+      <c r="H2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="M2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="N2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="O2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="P2" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="Q2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="R2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
+      <c r="S2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T2" s="13"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A3" s="2"/>
@@ -829,11 +890,15 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C3:C100000">

</xml_diff>